<commit_message>
Weekly camera events update (Samsara API)
</commit_message>
<xml_diff>
--- a/camera_events.xlsx
+++ b/camera_events.xlsx
@@ -496,24 +496,20 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>07/31/2026 12:01:49 PM</t>
+          <t>08/06/2026 6:47:11 PM</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Truck 13</t>
+          <t>Truck 8</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Josh Caldwell</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Full fleet , Light Duty</t>
-        </is>
-      </c>
+          <t>Kendall Mckerley</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t xml:space="preserve">Current Trucks, Full fleet </t>
@@ -521,7 +517,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Harsh Brake</t>
+          <t>Mobile Usage</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -535,32 +531,30 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="n">
-        <v>0.535</v>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>07/30/2026 3:53:18 PM</t>
+          <t>08/06/2026 10:52:41 AM</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Truck 3</t>
+          <t>Truck 32</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Mark Gwin</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Full fleet </t>
-        </is>
-      </c>
+          <t>Josh Gregory</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t xml:space="preserve">Current Trucks, Full fleet </t>
@@ -568,7 +562,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Ran Red Light</t>
+          <t>Mobile Usage</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -592,22 +586,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>07/27/2026 5:28:21 PM</t>
+          <t>08/04/2026 4:21:54 PM</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SV1</t>
+          <t>Truck 12</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Peyton Birchfield</t>
+          <t>Ben Mcgough</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Full fleet </t>
+          <t>Full fleet , Light Duty</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -617,7 +611,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Harsh Brake</t>
+          <t>Mobile Usage</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -631,25 +625,27 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="n">
-        <v>0.736</v>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>07/27/2026 7:08:38 AM</t>
+          <t>08/03/2026 7:28:46 PM</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Truck 12</t>
+          <t>Truck 1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Ben Mcgough</t>
+          <t>John Arnold</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -664,7 +660,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Mobile Usage</t>
+          <t>Rolling Stop</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -688,17 +684,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>07/26/2026 10:40:27 AM</t>
+          <t>07/31/2026 12:01:49 PM</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Truck 12</t>
+          <t>Truck 13</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Ben Mcgough</t>
+          <t>Josh Caldwell</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -713,7 +709,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Inattentive Driving</t>
+          <t>Harsh Brake</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -727,32 +723,30 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="N6" t="n">
+        <v>0.535</v>
       </c>
       <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>07/26/2026 8:12:01 AM</t>
+          <t>07/30/2026 3:53:18 PM</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Truck 6</t>
+          <t>Truck 3</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Robert Bailey</t>
+          <t>Mark Gwin</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Full fleet , Light Duty</t>
+          <t xml:space="preserve">Full fleet </t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -762,7 +756,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Harsh Turn</t>
+          <t>Ran Red Light</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -776,28 +770,34 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="n">
-        <v>0.585</v>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>07/23/2026 9:24:45 AM</t>
+          <t>07/27/2026 5:28:21 PM</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Truck 26</t>
+          <t>SV1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Kendall Mckerley</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
+          <t>Peyton Birchfield</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Full fleet </t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
           <t xml:space="preserve">Current Trucks, Full fleet </t>
@@ -805,7 +805,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Mobile Usage</t>
+          <t>Harsh Brake</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -819,22 +819,20 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="N8" t="n">
+        <v>0.736</v>
       </c>
       <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>07/22/2026 2:46:36 PM</t>
+          <t>07/27/2026 7:08:38 AM</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Truck 1</t>
+          <t>Truck 12</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -878,22 +876,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07/22/2026 8:57:05 AM</t>
+          <t>07/26/2026 10:40:27 AM</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Truck 32</t>
+          <t>Truck 12</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Nick Whitaker</t>
+          <t>Ben Mcgough</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Full fleet , Heavy Duty</t>
+          <t>Full fleet , Light Duty</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -903,7 +901,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Rolling Stop</t>
+          <t>Inattentive Driving</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -927,17 +925,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07/22/2026 1:42:12 AM</t>
+          <t>07/26/2026 8:12:01 AM</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Truck 1</t>
+          <t>Truck 6</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Chris Mcconnell</t>
+          <t>Robert Bailey</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -952,7 +950,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Drowsy</t>
+          <t>Harsh Turn</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -966,34 +964,28 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="N11" t="n">
+        <v>0.585</v>
       </c>
       <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07/21/2026 10:34:37 AM</t>
+          <t>07/23/2026 9:24:45 AM</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Truck 1</t>
+          <t>Truck 26</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Chris Mcconnell</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Full fleet , Light Duty</t>
-        </is>
-      </c>
+          <t>Kendall Mckerley</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t xml:space="preserve">Current Trucks, Full fleet </t>
@@ -1001,7 +993,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Inattentive Driving</t>
+          <t>Mobile Usage</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -1025,20 +1017,24 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07/20/2026 4:24:06 PM</t>
+          <t>07/22/2026 2:46:36 PM</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Truck 32</t>
+          <t>Truck 1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Josh Gregory</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr"/>
+          <t>Ben Mcgough</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Full fleet , Light Duty</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr">
         <is>
           <t xml:space="preserve">Current Trucks, Full fleet </t>
@@ -1046,7 +1042,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Harsh Brake</t>
+          <t>Mobile Usage</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
@@ -1060,30 +1056,32 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" t="n">
-        <v>0.798</v>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>07/20/2026 2:59:26 PM</t>
+          <t>07/22/2026 8:57:05 AM</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Truck 12</t>
+          <t>Truck 32</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Ben Mcgough</t>
+          <t>Nick Whitaker</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Full fleet , Light Duty</t>
+          <t>Full fleet , Heavy Duty</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1093,7 +1091,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Following Distance</t>
+          <t>Rolling Stop</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1107,25 +1105,27 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" t="n">
-        <v>0.538</v>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>07/19/2026 5:07:21 PM</t>
+          <t>07/22/2026 1:42:12 AM</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Truck 13</t>
+          <t>Truck 1</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Josh Caldwell</t>
+          <t>Chris Mcconnell</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Harsh Turn</t>
+          <t>Drowsy</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -1154,25 +1154,27 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
-      <c r="N15" t="n">
-        <v>0.47</v>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>07/16/2026 9:32:10 PM</t>
+          <t>07/21/2026 10:34:37 AM</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Truck 6</t>
+          <t>Truck 1</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Robert Bailey</t>
+          <t>Chris Mcconnell</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1187,7 +1189,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Crash</t>
+          <t>Inattentive Driving</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
@@ -1201,23 +1203,29 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" t="n">
-        <v>3.691</v>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>07/16/2026 8:50:56 AM</t>
+          <t>07/20/2026 4:24:06 PM</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Truck 12</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
+          <t>Truck 32</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Josh Gregory</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
@@ -1226,7 +1234,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>No Seat Belt</t>
+          <t>Harsh Brake</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
@@ -1240,30 +1248,32 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="N17" t="n">
+        <v>0.798</v>
       </c>
       <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>07/16/2026 1:50:44 AM</t>
+          <t>07/20/2026 2:59:26 PM</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Truck 22</t>
+          <t>Truck 12</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Josh Gregory</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
+          <t>Ben Mcgough</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Full fleet , Light Duty</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr">
         <is>
           <t xml:space="preserve">Current Trucks, Full fleet </t>
@@ -1271,7 +1281,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>No Seat Belt</t>
+          <t>Following Distance</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
@@ -1285,32 +1295,30 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="N18" t="n">
+        <v>0.538</v>
       </c>
       <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>07/15/2026 12:09:06 PM</t>
+          <t>07/19/2026 5:07:21 PM</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Truck 3</t>
+          <t>Truck 13</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Bryan Deshotel</t>
+          <t>Josh Caldwell</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Full fleet </t>
+          <t>Full fleet , Light Duty</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1320,7 +1328,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Inattentive Driving</t>
+          <t>Harsh Turn</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
@@ -1334,27 +1342,25 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="N19" t="n">
+        <v>0.47</v>
       </c>
       <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>07/14/2026 9:10:53 AM</t>
+          <t>07/16/2026 9:32:10 PM</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Truck 12</t>
+          <t>Truck 6</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Ben Mcgough</t>
+          <t>Robert Bailey</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1369,7 +1375,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Inattentive Driving</t>
+          <t>Crash</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
@@ -1383,34 +1389,24 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="N20" t="n">
+        <v>3.691</v>
       </c>
       <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07/09/2026 5:35:48 PM</t>
+          <t>07/16/2026 8:50:56 AM</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>SV1</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Peyton Birchfield</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Full fleet </t>
-        </is>
-      </c>
+          <t>Truck 12</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t xml:space="preserve">Current Trucks, Full fleet </t>
@@ -1418,7 +1414,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Harsh Turn</t>
+          <t>No Seat Belt</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
@@ -1432,32 +1428,30 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
-      <c r="N21" t="n">
-        <v>0.586</v>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>07/07/2026 4:24:46 PM</t>
+          <t>07/16/2026 1:50:44 AM</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Truck 8</t>
+          <t>Truck 22</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Robert Bailey</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Full fleet , Light Duty</t>
-        </is>
-      </c>
+          <t>Josh Gregory</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t xml:space="preserve">Current Trucks, Full fleet </t>
@@ -1465,7 +1459,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Mobile Usage</t>
+          <t>No Seat Belt</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1489,20 +1483,24 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>07/06/2026 1:15:36 AM</t>
+          <t>07/15/2026 12:09:06 PM</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>SV1</t>
+          <t>Truck 3</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Donald White</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr"/>
+          <t>Bryan Deshotel</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Full fleet </t>
+        </is>
+      </c>
       <c r="E23" t="inlineStr">
         <is>
           <t xml:space="preserve">Current Trucks, Full fleet </t>
@@ -1510,7 +1508,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Drowsy</t>
+          <t>Inattentive Driving</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
@@ -1534,22 +1532,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>07/03/2026 1:27:36 AM</t>
+          <t>07/14/2026 9:10:53 AM</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SV1</t>
+          <t>Truck 12</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Peyton Birchfield</t>
+          <t>Ben Mcgough</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Full fleet </t>
+          <t>Full fleet , Light Duty</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1559,7 +1557,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Drowsy</t>
+          <t>Inattentive Driving</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
@@ -1583,7 +1581,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>07/02/2026 7:36:53 AM</t>
+          <t>07/09/2026 5:35:48 PM</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1608,7 +1606,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Forward Collision Warning</t>
+          <t>Harsh Turn</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
@@ -1622,32 +1620,30 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="N25" t="n">
+        <v>0.586</v>
       </c>
       <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>07/01/2026 11:21:32 AM</t>
+          <t>07/07/2026 4:24:46 PM</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Truck 26</t>
+          <t>Truck 8</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Daniel Vanwinterswyk</t>
+          <t>Robert Bailey</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Full fleet , Heavy Duty</t>
+          <t>Full fleet , Light Duty</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1657,7 +1653,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Drowsy</t>
+          <t>Mobile Usage</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
@@ -1681,24 +1677,20 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06/30/2026 10:56:28 AM</t>
+          <t>07/06/2026 1:15:36 AM</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Truck 26</t>
+          <t>SV1</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Nick Whitaker</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Full fleet , Heavy Duty</t>
-        </is>
-      </c>
+          <t>Donald White</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
           <t xml:space="preserve">Current Trucks, Full fleet </t>
@@ -1706,7 +1698,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Rolling Stop</t>
+          <t>Drowsy</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
@@ -1730,7 +1722,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>06/25/2026 9:42:46 AM</t>
+          <t>07/03/2026 1:27:36 AM</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1755,7 +1747,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Camera Obstruction</t>
+          <t>Drowsy</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
@@ -1779,22 +1771,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>06/24/2026 4:25:18 PM</t>
+          <t>07/02/2026 7:36:53 AM</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Truck 45</t>
+          <t>SV1</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Will Ordoyne</t>
+          <t>Peyton Birchfield</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Full fleet , Heavy Duty</t>
+          <t xml:space="preserve">Full fleet </t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1804,7 +1796,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Drowsy</t>
+          <t>Forward Collision Warning</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
@@ -1828,7 +1820,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>06/23/2026 3:35:05 PM</t>
+          <t>07/01/2026 11:21:32 AM</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1838,7 +1830,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Nick Whitaker</t>
+          <t>Daniel Vanwinterswyk</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1853,7 +1845,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Harsh Brake</t>
+          <t>Drowsy</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
@@ -1867,30 +1859,32 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" t="n">
-        <v>0.528</v>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>06/23/2026 6:54:31 AM</t>
+          <t>06/30/2026 10:56:28 AM</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Truck 12</t>
+          <t>Truck 26</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Ben Mcgough</t>
+          <t>Nick Whitaker</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Full fleet , Light Duty</t>
+          <t>Full fleet , Heavy Duty</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1900,7 +1894,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Drowsy</t>
+          <t>Rolling Stop</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
@@ -1924,22 +1918,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>06/22/2026 9:11:54 PM</t>
+          <t>06/25/2026 9:42:46 AM</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Truck 12</t>
+          <t>SV1</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Will Ordoyne</t>
+          <t>Peyton Birchfield</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Full fleet , Heavy Duty</t>
+          <t xml:space="preserve">Full fleet </t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1949,7 +1943,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Harsh Turn</t>
+          <t>Camera Obstruction</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
@@ -1963,30 +1957,32 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" t="n">
-        <v>0.541</v>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>06/18/2026 6:18:24 PM</t>
+          <t>06/24/2026 4:25:18 PM</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Truck 6</t>
+          <t>Truck 45</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Robert Bailey</t>
+          <t>Will Ordoyne</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Full fleet , Light Duty</t>
+          <t>Full fleet , Heavy Duty</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1996,7 +1992,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Rolling Stop</t>
+          <t>Drowsy</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
@@ -2020,20 +2016,24 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06/17/2026 2:01:08 PM</t>
+          <t>06/23/2026 3:35:05 PM</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Truck 32</t>
+          <t>Truck 26</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Josh Gregory</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr"/>
+          <t>Nick Whitaker</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Full fleet , Heavy Duty</t>
+        </is>
+      </c>
       <c r="E34" t="inlineStr">
         <is>
           <t xml:space="preserve">Current Trucks, Full fleet </t>
@@ -2041,7 +2041,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Following Distance</t>
+          <t>Harsh Brake</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
@@ -2055,32 +2055,30 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="N34" t="n">
+        <v>0.528</v>
       </c>
       <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>06/15/2026 4:15:12 PM</t>
+          <t>06/23/2026 6:54:31 AM</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Truck 32</t>
+          <t>Truck 12</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Daniel Vanwinterswyk</t>
+          <t>Ben Mcgough</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Full fleet , Heavy Duty</t>
+          <t>Full fleet , Light Duty</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2096,7 +2094,7 @@
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Coached</t>
+          <t>Needs Coaching</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
@@ -2114,7 +2112,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>06/15/2026 8:32:09 AM</t>
+          <t>06/22/2026 9:11:54 PM</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2124,12 +2122,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Ben Mcgough</t>
+          <t>Will Ordoyne</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Full fleet , Light Duty</t>
+          <t>Full fleet , Heavy Duty</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2139,7 +2137,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Inattentive Driving</t>
+          <t>Harsh Turn</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
@@ -2153,32 +2151,30 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="N36" t="n">
+        <v>0.541</v>
       </c>
       <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>06/12/2026 10:25:32 PM</t>
+          <t>06/18/2026 6:18:24 PM</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Truck 3</t>
+          <t>Truck 6</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Mark Gwin</t>
+          <t>Robert Bailey</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Full fleet </t>
+          <t>Full fleet , Light Duty</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2188,7 +2184,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Mobile Usage</t>
+          <t>Rolling Stop</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
@@ -2212,12 +2208,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>06/12/2026 1:46:41 PM</t>
+          <t>06/17/2026 2:01:08 PM</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Truck 22</t>
+          <t>Truck 32</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2233,7 +2229,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Mobile Usage</t>
+          <t>Following Distance</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
@@ -2257,22 +2253,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>06/11/2026 3:36:21 PM</t>
+          <t>06/15/2026 4:15:12 PM</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Truck 8</t>
+          <t>Truck 32</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Chris Mcconnell</t>
+          <t>Daniel Vanwinterswyk</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Full fleet , Light Duty</t>
+          <t>Full fleet , Heavy Duty</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2282,13 +2278,13 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Inattentive Driving</t>
+          <t>Drowsy</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Needs Coaching</t>
+          <t>Coached</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
@@ -2306,16 +2302,24 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>06/11/2026 11:14:55 AM</t>
+          <t>06/15/2026 8:32:09 AM</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>E-1</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
+          <t>Truck 12</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Ben Mcgough</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Full fleet , Light Duty</t>
+        </is>
+      </c>
       <c r="E40" t="inlineStr">
         <is>
           <t xml:space="preserve">Current Trucks, Full fleet </t>
@@ -2323,7 +2327,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Mobile Usage</t>
+          <t>Inattentive Driving</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
@@ -2347,17 +2351,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>06/10/2026 3:29:55 PM</t>
+          <t>06/12/2026 10:25:32 PM</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Truck 7</t>
+          <t>Truck 3</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Bryan Deshotel</t>
+          <t>Mark Gwin</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2372,7 +2376,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Crash</t>
+          <t>Mobile Usage</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
@@ -2386,32 +2390,30 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
-      <c r="N41" t="n">
-        <v>5.497</v>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06/10/2026 6:19:44 AM</t>
+          <t>06/12/2026 1:46:41 PM</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SV1</t>
+          <t>Truck 22</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Peyton Birchfield</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Full fleet </t>
-        </is>
-      </c>
+          <t>Josh Gregory</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
           <t xml:space="preserve">Current Trucks, Full fleet </t>
@@ -2443,16 +2445,24 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06/08/2026 3:02:41 PM</t>
+          <t>06/11/2026 3:36:21 PM</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>E-1</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
+          <t>Truck 8</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Chris Mcconnell</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Full fleet , Light Duty</t>
+        </is>
+      </c>
       <c r="E43" t="inlineStr">
         <is>
           <t xml:space="preserve">Current Trucks, Full fleet </t>
@@ -2460,7 +2470,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Mobile Usage</t>
+          <t>Inattentive Driving</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
@@ -2484,24 +2494,16 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06/07/2026 3:36:18 AM</t>
+          <t>06/11/2026 11:14:55 AM</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SV1</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Peyton Birchfield</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Full fleet </t>
-        </is>
-      </c>
+          <t>E-1</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
           <t xml:space="preserve">Current Trucks, Full fleet </t>
@@ -2509,7 +2511,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Drowsy</t>
+          <t>Mobile Usage</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
@@ -2533,22 +2535,22 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06/01/2026 8:11:54 PM</t>
+          <t>06/10/2026 3:29:55 PM</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Truck 12</t>
+          <t>Truck 7</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Josh Caldwell</t>
+          <t>Bryan Deshotel</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Full fleet , Light Duty</t>
+          <t xml:space="preserve">Full fleet </t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2558,7 +2560,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Inattentive Driving</t>
+          <t>Crash</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
@@ -2572,26 +2574,32 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="N45" t="n">
+        <v>5.497</v>
       </c>
       <c r="O45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>05/28/2026 5:38:57 PM</t>
+          <t>06/10/2026 6:19:44 AM</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Truck 12</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
+          <t>SV1</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Peyton Birchfield</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Full fleet </t>
+        </is>
+      </c>
       <c r="E46" t="inlineStr">
         <is>
           <t xml:space="preserve">Current Trucks, Full fleet </t>
@@ -2599,7 +2607,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>No Seat Belt</t>
+          <t>Mobile Usage</t>
         </is>
       </c>
       <c r="G46" t="inlineStr"/>
@@ -2623,12 +2631,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>05/28/2026 1:42:30 PM</t>
+          <t>06/08/2026 3:02:41 PM</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Truck 7</t>
+          <t>E-1</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -2640,7 +2648,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>No Seat Belt</t>
+          <t>Mobile Usage</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
@@ -2664,22 +2672,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>05/26/2026 2:44:39 PM</t>
+          <t>06/07/2026 3:36:18 AM</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Truck 8</t>
+          <t>SV1</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Chris Mcconnell</t>
+          <t>Peyton Birchfield</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Full fleet , Light Duty</t>
+          <t xml:space="preserve">Full fleet </t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2689,7 +2697,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Harsh Brake</t>
+          <t>Drowsy</t>
         </is>
       </c>
       <c r="G48" t="inlineStr"/>
@@ -2703,28 +2711,34 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
-      <c r="N48" t="n">
-        <v>0.484</v>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>05/26/2026 2:13:56 PM</t>
+          <t>06/01/2026 8:11:54 PM</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Truck 22</t>
+          <t>Truck 12</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Josh Gregory</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr"/>
+          <t>Josh Caldwell</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Full fleet , Light Duty</t>
+        </is>
+      </c>
       <c r="E49" t="inlineStr">
         <is>
           <t xml:space="preserve">Current Trucks, Full fleet </t>
@@ -2732,7 +2746,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Harsh Brake</t>
+          <t>Inattentive Driving</t>
         </is>
       </c>
       <c r="G49" t="inlineStr"/>
@@ -2746,32 +2760,26 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr"/>
-      <c r="N49" t="n">
-        <v>0.502</v>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>05/23/2026 1:29:29 AM</t>
+          <t>05/28/2026 5:38:57 PM</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SV1</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Peyton Birchfield</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Full fleet </t>
-        </is>
-      </c>
+          <t>Truck 12</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
           <t xml:space="preserve">Current Trucks, Full fleet </t>
@@ -2779,7 +2787,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Drowsy</t>
+          <t>No Seat Belt</t>
         </is>
       </c>
       <c r="G50" t="inlineStr"/>
@@ -2803,24 +2811,16 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>05/19/2026 10:16:58 PM</t>
+          <t>05/28/2026 1:42:30 PM</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Truck 6</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Robert Bailey</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Full fleet , Light Duty</t>
-        </is>
-      </c>
+          <t>Truck 7</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
           <t xml:space="preserve">Current Trucks, Full fleet </t>
@@ -2852,22 +2852,22 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>05/19/2026 4:22:07 AM</t>
+          <t>05/26/2026 2:44:39 PM</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Truck 3</t>
+          <t>Truck 8</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Mark Gwin</t>
+          <t>Chris Mcconnell</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Full fleet </t>
+          <t>Full fleet , Light Duty</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2877,7 +2877,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Drowsy</t>
+          <t>Harsh Brake</t>
         </is>
       </c>
       <c r="G52" t="inlineStr"/>
@@ -2891,34 +2891,28 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="N52" t="n">
+        <v>0.484</v>
       </c>
       <c r="O52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>05/10/2026 11:46:38 PM</t>
+          <t>05/26/2026 2:13:56 PM</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Truck 8</t>
+          <t>Truck 22</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Chris Mcconnell</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Full fleet , Light Duty</t>
-        </is>
-      </c>
+          <t>Josh Gregory</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
           <t xml:space="preserve">Current Trucks, Full fleet </t>
@@ -2941,23 +2935,31 @@
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr"/>
       <c r="N53" t="n">
-        <v>0.9379999999999999</v>
+        <v>0.502</v>
       </c>
       <c r="O53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>05/08/2026 6:49:37 AM</t>
+          <t>05/23/2026 1:29:29 AM</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Truck 7</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
+          <t>SV1</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Peyton Birchfield</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Full fleet </t>
+        </is>
+      </c>
       <c r="E54" t="inlineStr">
         <is>
           <t xml:space="preserve">Current Trucks, Full fleet </t>
@@ -2965,7 +2967,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Harsh Turn</t>
+          <t>Drowsy</t>
         </is>
       </c>
       <c r="G54" t="inlineStr"/>
@@ -2979,28 +2981,34 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr"/>
-      <c r="N54" t="n">
-        <v>0.486</v>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>05/06/2026 10:32:16 AM</t>
+          <t>05/19/2026 10:16:58 PM</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>SV1</t>
+          <t>Truck 6</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Donald White</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr"/>
+          <t>Robert Bailey</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Full fleet , Light Duty</t>
+        </is>
+      </c>
       <c r="E55" t="inlineStr">
         <is>
           <t xml:space="preserve">Current Trucks, Full fleet </t>
@@ -3032,22 +3040,22 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>05/06/2026 8:26:47 AM</t>
+          <t>05/19/2026 4:22:07 AM</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Truck 26</t>
+          <t>Truck 3</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Chico Leone</t>
+          <t>Mark Gwin</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Full fleet , Heavy Duty</t>
+          <t xml:space="preserve">Full fleet </t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3057,7 +3065,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Following Distance</t>
+          <t>Drowsy</t>
         </is>
       </c>
       <c r="G56" t="inlineStr"/>

</xml_diff>